<commit_message>
add application.properties file and also add runtest command file to run the test
</commit_message>
<xml_diff>
--- a/appium/phone_numbers.xlsx
+++ b/appium/phone_numbers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,50 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>btkral-wd@example.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>507067387</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>نوره</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>كانو</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>hal-hsyn@example.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>531980950</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>جنى</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>آل العسكري</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>jal-khdyr@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>